<commit_message>
docs: adiciona demonstracao em GIF da execucao no topo do README
</commit_message>
<xml_diff>
--- a/dados/resultados/controle_conciliacao.xlsx
+++ b/dados/resultados/controle_conciliacao.xlsx
@@ -319,7 +319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="16.59765625" customWidth="1" min="1" max="1"/>
@@ -784,6 +784,68 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-05T06:21:12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FAT-2026-00192</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PO-2026-0421</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>12.345.678/0001-90</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NovaCore Tecnologia Ltda</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1750.00</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1750</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FATURA_DUPLICADA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Fatura já processada anteriormente</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>jeova</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>